<commit_message>
First draft of figures finished
</commit_message>
<xml_diff>
--- a/auxiliary_data/GHE.xlsx
+++ b/auxiliary_data/GHE.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meurerst\git\anonymization-review-fork\auxiliary_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65681CBE-4E53-47BE-9A84-C487E0AF171A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4015E3D5-FA11-4170-83E4-3ECA1EC9E232}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="8304" windowHeight="4512" activeTab="2" xr2:uid="{34061D47-98F9-43FC-9E51-B12C99A01ED8}"/>
   </bookViews>
   <sheets>
     <sheet name="Source" sheetId="1" r:id="rId1"/>
     <sheet name="Statistics" sheetId="2" r:id="rId2"/>
-    <sheet name="Tabelle4" sheetId="4" r:id="rId3"/>
-    <sheet name="Mapping" sheetId="3" r:id="rId4"/>
+    <sheet name="Total Deaths" sheetId="5" r:id="rId3"/>
+    <sheet name="Tabelle4" sheetId="4" r:id="rId4"/>
+    <sheet name="Mapping" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="44">
   <si>
     <t>Disease area</t>
   </si>
@@ -157,6 +158,9 @@
   </si>
   <si>
     <t>Deaths (High-income economies)</t>
+  </si>
+  <si>
+    <t>other</t>
   </si>
 </sst>
 </file>
@@ -2533,6 +2537,253 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{065BF169-F3E8-4041-9E16-95D706A4263B}">
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>266</v>
+      </c>
+      <c r="E2" s="4">
+        <v>4747</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="4">
+        <v>2860</v>
+      </c>
+      <c r="E3" s="4">
+        <v>12566</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="D4" s="4">
+        <v>3214</v>
+      </c>
+      <c r="E4" s="4">
+        <v>6641</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5">
+        <v>892</v>
+      </c>
+      <c r="E5" s="4">
+        <v>3013</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="4">
+        <v>1367</v>
+      </c>
+      <c r="E6" s="4">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7">
+        <v>9</v>
+      </c>
+      <c r="D7" s="4">
+        <v>4445</v>
+      </c>
+      <c r="E7" s="4">
+        <v>14652</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8">
+        <v>15</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9">
+        <v>16</v>
+      </c>
+      <c r="D9">
+        <v>27</v>
+      </c>
+      <c r="E9" s="4">
+        <v>1894</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>8</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11">
+        <v>11</v>
+      </c>
+      <c r="D11">
+        <v>621</v>
+      </c>
+      <c r="E11" s="4">
+        <v>1860</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>12</v>
+      </c>
+      <c r="D12">
+        <v>32</v>
+      </c>
+      <c r="E12">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>72</v>
+      </c>
+      <c r="E13">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>17</v>
+      </c>
+      <c r="D14">
+        <v>39</v>
+      </c>
+      <c r="E14">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>18</v>
+      </c>
+      <c r="D15">
+        <v>2</v>
+      </c>
+      <c r="E15">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16">
+        <v>20</v>
+      </c>
+      <c r="D16">
+        <v>721</v>
+      </c>
+      <c r="E16" s="4">
+        <v>3719</v>
+      </c>
+    </row>
+    <row r="20" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C20" t="s">
+        <v>43</v>
+      </c>
+      <c r="D20">
+        <f>SUM(D8:D16)</f>
+        <v>1517</v>
+      </c>
+      <c r="E20">
+        <f>SUM(E8:E16)</f>
+        <v>8387</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BA9A350-9689-4A97-964A-DDD3A3242BBA}">
   <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2729,7 +2980,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A9AFF55-C9DE-4299-B06F-E3BAFF9A2D24}">
   <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Added labels in figure 1b
</commit_message>
<xml_diff>
--- a/auxiliary_data/GHE.xlsx
+++ b/auxiliary_data/GHE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meurerst\git\anonymization-review-fork\auxiliary_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4015E3D5-FA11-4170-83E4-3ECA1EC9E232}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D1DE666-772B-4AB6-84F1-AD7E900E7925}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="8304" windowHeight="4512" activeTab="2" xr2:uid="{34061D47-98F9-43FC-9E51-B12C99A01ED8}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="8304" windowHeight="4512" activeTab="1" xr2:uid="{34061D47-98F9-43FC-9E51-B12C99A01ED8}"/>
   </bookViews>
   <sheets>
     <sheet name="Source" sheetId="1" r:id="rId1"/>
@@ -1307,7 +1307,10 @@
         <f>S2*100/S$18</f>
         <v>1.8267976100542545</v>
       </c>
-      <c r="Z2" s="4"/>
+      <c r="Z2" s="4">
+        <f>R2+S2</f>
+        <v>5012.5588293872788</v>
+      </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -1380,7 +1383,10 @@
         <f t="shared" ref="X3:X16" si="2">S3*100/S$18</f>
         <v>19.641508138177322</v>
       </c>
-      <c r="Z3" s="4"/>
+      <c r="Z3" s="4">
+        <f t="shared" ref="Z3:Z16" si="3">R3+S3</f>
+        <v>15426.145700484121</v>
+      </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -1453,7 +1459,10 @@
         <f t="shared" si="2"/>
         <v>22.072659844790881</v>
       </c>
-      <c r="Z4" s="4"/>
+      <c r="Z4" s="4">
+        <f t="shared" si="3"/>
+        <v>9854.9727741605675</v>
+      </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
@@ -1526,7 +1535,10 @@
         <f t="shared" si="2"/>
         <v>6.1259528878511089</v>
       </c>
-      <c r="Z5" s="4"/>
+      <c r="Z5" s="4">
+        <f t="shared" si="3"/>
+        <v>3904.9281331834059</v>
+      </c>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -1599,7 +1611,10 @@
         <f t="shared" si="2"/>
         <v>9.3880914772337061</v>
       </c>
-      <c r="Z6" s="4"/>
+      <c r="Z6" s="4">
+        <f t="shared" si="3"/>
+        <v>2869.5437717172954</v>
+      </c>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -1668,7 +1683,10 @@
         <f t="shared" si="2"/>
         <v>30.526749536432938</v>
       </c>
-      <c r="Z7" s="4"/>
+      <c r="Z7" s="4">
+        <f t="shared" si="3"/>
+        <v>19097.172532221881</v>
+      </c>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -1737,7 +1755,10 @@
         <f t="shared" si="2"/>
         <v>1.3735320376347778E-2</v>
       </c>
-      <c r="Z8" s="4"/>
+      <c r="Z8" s="4">
+        <f t="shared" si="3"/>
+        <v>257.51987623515083</v>
+      </c>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -1806,7 +1827,10 @@
         <f t="shared" si="2"/>
         <v>0.185426825080695</v>
       </c>
-      <c r="Z9" s="4"/>
+      <c r="Z9" s="4">
+        <f t="shared" si="3"/>
+        <v>1921.0733932876117</v>
+      </c>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
@@ -1875,7 +1899,10 @@
         <f t="shared" si="2"/>
         <v>6.8676601881738891E-3</v>
       </c>
-      <c r="Z10" s="4"/>
+      <c r="Z10" s="4">
+        <f t="shared" si="3"/>
+        <v>1.301531804068309</v>
+      </c>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
@@ -1948,7 +1975,10 @@
         <f t="shared" si="2"/>
         <v>4.2648169768559852</v>
       </c>
-      <c r="Z11" s="4"/>
+      <c r="Z11" s="4">
+        <f t="shared" si="3"/>
+        <v>2481.2429442772404</v>
+      </c>
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -2017,7 +2047,10 @@
         <f t="shared" si="2"/>
         <v>0.21976512602156445</v>
       </c>
-      <c r="Z12" s="4"/>
+      <c r="Z12" s="4">
+        <f t="shared" si="3"/>
+        <v>91.556869943406667</v>
+      </c>
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -2086,7 +2119,10 @@
         <f t="shared" si="2"/>
         <v>0.49447153354852003</v>
       </c>
-      <c r="Z13" s="4"/>
+      <c r="Z13" s="4">
+        <f t="shared" si="3"/>
+        <v>161.33824112132322</v>
+      </c>
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
@@ -2155,7 +2191,10 @@
         <f t="shared" si="2"/>
         <v>0.26783874733878166</v>
       </c>
-      <c r="Z14" s="4"/>
+      <c r="Z14" s="4">
+        <f t="shared" si="3"/>
+        <v>523.03897810680826</v>
+      </c>
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
@@ -2224,7 +2263,10 @@
         <f t="shared" si="2"/>
         <v>1.3735320376347778E-2</v>
       </c>
-      <c r="Z15" s="4"/>
+      <c r="Z15" s="4">
+        <f t="shared" si="3"/>
+        <v>26.776747911121088</v>
+      </c>
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
@@ -2297,7 +2339,10 @@
         <f t="shared" si="2"/>
         <v>4.9515829956733741</v>
       </c>
-      <c r="Z16" s="4"/>
+      <c r="Z16" s="4">
+        <f t="shared" si="3"/>
+        <v>4439.7310480912502</v>
+      </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
@@ -2353,23 +2398,23 @@
         <v>5084.2957529925952</v>
       </c>
       <c r="L18">
-        <f t="shared" ref="L18:S18" si="3">SUM(L2:L16)</f>
+        <f t="shared" ref="L18:S18" si="4">SUM(L2:L16)</f>
         <v>23131.385085728703</v>
       </c>
       <c r="M18">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>23292.220533211232</v>
       </c>
       <c r="N18">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>14561.437776354171</v>
       </c>
       <c r="R18">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>51507.90137193253</v>
       </c>
       <c r="S18">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>14561</v>
       </c>
     </row>

</xml_diff>